<commit_message>
Include Altair BASIC 2.0
</commit_message>
<xml_diff>
--- a/sw/Languajes/Basic/Microsoft Basic/MS Basic TimeLine.xlsx
+++ b/sw/Languajes/Basic/Microsoft Basic/MS Basic TimeLine.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>Altair</t>
   </si>
@@ -253,6 +253,9 @@
   <si>
     <t>EPSON MultiFonts 
 BASIC 1.3 (QX10)</t>
+  </si>
+  <si>
+    <t>BASIC 8K 2.0</t>
   </si>
 </sst>
 </file>
@@ -637,7 +640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.1796875" style="1"/>
@@ -709,367 +712,373 @@
       </c>
       <c r="C3" s="6"/>
     </row>
-    <row r="4" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
-        <v>2</v>
+        <v>77</v>
       </c>
       <c r="C4" s="6"/>
     </row>
     <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="6"/>
     </row>
     <row r="6" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="6"/>
     </row>
     <row r="7" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>7</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="C7" s="6"/>
     </row>
     <row r="8" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>1976</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="6"/>
     </row>
     <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
+        <v>1976</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>1977</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>1978</v>
-      </c>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>1978</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
         <v>1979</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F15" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="E15" s="3" t="s">
+    <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="E16" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
         <v>1980</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F17" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="D17" s="3" t="s">
+    <row r="18" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="D18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
+    <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
         <v>1981</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="G19" s="5" t="s">
+    <row r="20" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="G20" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
+    <row r="21" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
         <v>1982</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H21" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="5" t="s">
+    <row r="22" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D22" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="1">
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="1">
         <v>1983</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="G23" s="5" t="s">
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="G24" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="G24" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="G25" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="G26" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
         <v>1984</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
+    <row r="28" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
         <v>1985</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="H29" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H29" s="3" t="s">
+    <row r="30" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H30" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
+    <row r="31" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
         <v>1986</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G31" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
         <v>1987</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H33" s="3" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="H33" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="H34" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="H35" s="3" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>1988</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>1989</v>
+        <v>1988</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>1990</v>
+        <v>1989</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>1991</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>70</v>
+        <v>1990</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
+        <v>1991</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="1">
         <v>1992</v>
       </c>
-      <c r="I39" s="3" t="s">
+      <c r="I40" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="1">
         <v>1993</v>
       </c>
-      <c r="I40" s="3" t="s">
+      <c r="I41" s="3" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <v>1994</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
-        <v>1995</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>74</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
-        <v>1996</v>
+        <v>1995</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
-        <v>1997</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>75</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
+        <v>1997</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46" s="1">
         <v>1998</v>
       </c>
-      <c r="I45" s="3" t="s">
+      <c r="I46" s="3" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>